<commit_message>
Business case: commit to every site, no phased funding; 1% question; intangibles wording; template rollout sheet
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Y4SNSUs71veJ37BenGhXFE
</commit_message>
<xml_diff>
--- a/public/downloads/shopfloor-matters-business-case-template.xlsx
+++ b/public/downloads/shopfloor-matters-business-case-template.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Benefits" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="Costs" sheetId="4" state="visible" r:id="rId6"/>
     <sheet name="Cash flow" sheetId="5" state="visible" r:id="rId7"/>
-    <sheet name="Phasing" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="Rollout" sheetId="6" state="visible" r:id="rId8"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -64,7 +64,7 @@
     <t xml:space="preserve">3. Realistic costs and timeline, including your own people, not just licences and services (Costs).</t>
   </si>
   <si>
-    <t xml:space="preserve">4. How the risk is managed: phases, measures and decision points (Phasing).</t>
+    <t xml:space="preserve">4. How the risk is managed: a clear rollout plan across every site, with milestones and measures (Rollout).</t>
   </si>
   <si>
     <t xml:space="preserve">How to use it:</t>
@@ -73,7 +73,7 @@
     <t xml:space="preserve">Fill in Baseline with numbers finance will recognise. Set deliberately modest improvements on Benefits. Fill in every cost line, then read Cash flow.</t>
   </si>
   <si>
-    <t xml:space="preserve">Keep the first phase small: one line or one area. Let its results fund the next phase.</t>
+    <t xml:space="preserve">Make the case for every site as one programme: licences for all your sites, a template built on the first, and a clear plan for the rest.</t>
   </si>
   <si>
     <t xml:space="preserve">The example values describe a fictional mid-size site so you can see how it works. They are not a forecast. Replace them all.</t>
@@ -418,13 +418,13 @@
     <t xml:space="preserve">Every year you wait, this is what stays on the table.</t>
   </si>
   <si>
-    <t xml:space="preserve">Phasing: how the risk is managed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The section boards read most closely. Each phase has a scope, a measure and a decision point. The next phase only starts when the measure says so.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Phase</t>
+    <t xml:space="preserve">Rollout: how the risk is managed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The section boards read most closely. The programme covers every site. Each stage has a scope, a measure and a milestone, so progress is visible all the way.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stage</t>
   </si>
   <si>
     <t xml:space="preserve">Scope</t>
@@ -436,61 +436,61 @@
     <t xml:space="preserve">Success measure</t>
   </si>
   <si>
-    <t xml:space="preserve">Decision point</t>
+    <t xml:space="preserve">Milestone</t>
   </si>
   <si>
     <t xml:space="preserve">Owner</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Pilot</t>
-  </si>
-  <si>
-    <t xml:space="preserve">One line, production and quality</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4 to 6 months</t>
+    <t xml:space="preserve">1. First site</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The whole site, starting with production and quality</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6 to 9 months</t>
   </si>
   <si>
     <t xml:space="preserve">OEE up 3 points against baseline; scrap down 10%</t>
   </si>
   <si>
-    <t xml:space="preserve">Steering group review at month 6</t>
+    <t xml:space="preserve">First site live on every shift</t>
   </si>
   <si>
     <t xml:space="preserve">Operations director</t>
   </si>
   <si>
-    <t xml:space="preserve">2. Site</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Remaining lines on the site</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6 to 9 months</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Benefits on Benefits sheet reached at 80% ramp</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Before committing to site 2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Site lead</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3. Template</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Second site from the same template</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Go-live on time with under 10% local change</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Before wider roll-out</t>
+    <t xml:space="preserve">2. Template</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Standard processes, master data rules, KPIs and screens from the first site</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 to 3 months</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Template signed off by the centre of excellence</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Template ready for the next site</t>
   </si>
   <si>
     <t xml:space="preserve">Programme lead</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3. Remaining sites</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Every other site, from the same template</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4 to 6 months per site</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Go-live on time with under 10% local change; benefits on Benefits sheet reached</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Each site live on every shift</t>
   </si>
 </sst>
 </file>
@@ -658,108 +658,112 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="27">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="167" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1030,166 +1034,166 @@
   <dimension ref="A1:H19"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="2" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="2" style="1" width="14"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3"/>
-      <c r="H4" s="3"/>
+      <c r="B4" s="4"/>
+      <c r="C4" s="4"/>
+      <c r="D4" s="4"/>
+      <c r="E4" s="4"/>
+      <c r="F4" s="4"/>
+      <c r="G4" s="4"/>
+      <c r="H4" s="4"/>
     </row>
     <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="3"/>
-      <c r="C5" s="3"/>
-      <c r="D5" s="3"/>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
-      <c r="G5" s="3"/>
-      <c r="H5" s="3"/>
+      <c r="B5" s="4"/>
+      <c r="C5" s="4"/>
+      <c r="D5" s="4"/>
+      <c r="E5" s="4"/>
+      <c r="F5" s="4"/>
+      <c r="G5" s="4"/>
+      <c r="H5" s="4"/>
     </row>
     <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="3"/>
-      <c r="C6" s="3"/>
-      <c r="D6" s="3"/>
-      <c r="E6" s="3"/>
-      <c r="F6" s="3"/>
-      <c r="G6" s="3"/>
-      <c r="H6" s="3"/>
-    </row>
-    <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3" t="s">
+      <c r="B6" s="4"/>
+      <c r="C6" s="4"/>
+      <c r="D6" s="4"/>
+      <c r="E6" s="4"/>
+      <c r="F6" s="4"/>
+      <c r="G6" s="4"/>
+      <c r="H6" s="4"/>
+    </row>
+    <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="3"/>
-      <c r="C7" s="3"/>
-      <c r="D7" s="3"/>
-      <c r="E7" s="3"/>
-      <c r="F7" s="3"/>
-      <c r="G7" s="3"/>
-      <c r="H7" s="3"/>
+      <c r="B7" s="4"/>
+      <c r="C7" s="4"/>
+      <c r="D7" s="4"/>
+      <c r="E7" s="4"/>
+      <c r="F7" s="4"/>
+      <c r="G7" s="4"/>
+      <c r="H7" s="4"/>
     </row>
     <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2" t="s">
+      <c r="A8" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="2"/>
-      <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
-      <c r="E8" s="2"/>
-      <c r="F8" s="2"/>
-      <c r="G8" s="2"/>
-      <c r="H8" s="2"/>
+      <c r="B8" s="3"/>
+      <c r="C8" s="3"/>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
+      <c r="H8" s="3"/>
     </row>
     <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="s">
+      <c r="A9" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="3"/>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
-      <c r="E9" s="3"/>
-      <c r="F9" s="3"/>
-      <c r="G9" s="3"/>
-      <c r="H9" s="3"/>
-    </row>
-    <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="s">
+      <c r="B9" s="4"/>
+      <c r="C9" s="4"/>
+      <c r="D9" s="4"/>
+      <c r="E9" s="4"/>
+      <c r="F9" s="4"/>
+      <c r="G9" s="4"/>
+      <c r="H9" s="4"/>
+    </row>
+    <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="3"/>
-      <c r="C10" s="3"/>
-      <c r="D10" s="3"/>
-      <c r="E10" s="3"/>
-      <c r="F10" s="3"/>
-      <c r="G10" s="3"/>
-      <c r="H10" s="3"/>
+      <c r="B10" s="4"/>
+      <c r="C10" s="4"/>
+      <c r="D10" s="4"/>
+      <c r="E10" s="4"/>
+      <c r="F10" s="4"/>
+      <c r="G10" s="4"/>
+      <c r="H10" s="4"/>
     </row>
     <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3" t="s">
+      <c r="A11" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B11" s="3"/>
-      <c r="C11" s="3"/>
-      <c r="D11" s="3"/>
-      <c r="E11" s="3"/>
-      <c r="F11" s="3"/>
-      <c r="G11" s="3"/>
-      <c r="H11" s="3"/>
+      <c r="B11" s="4"/>
+      <c r="C11" s="4"/>
+      <c r="D11" s="4"/>
+      <c r="E11" s="4"/>
+      <c r="F11" s="4"/>
+      <c r="G11" s="4"/>
+      <c r="H11" s="4"/>
     </row>
     <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="3" t="s">
+      <c r="A12" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B12" s="3"/>
-      <c r="C12" s="3"/>
-      <c r="D12" s="3"/>
-      <c r="E12" s="3"/>
-      <c r="F12" s="3"/>
-      <c r="G12" s="3"/>
-      <c r="H12" s="3"/>
+      <c r="B12" s="4"/>
+      <c r="C12" s="4"/>
+      <c r="D12" s="4"/>
+      <c r="E12" s="4"/>
+      <c r="F12" s="4"/>
+      <c r="G12" s="4"/>
+      <c r="H12" s="4"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="4" t="s">
+      <c r="A14" s="5" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="5" t="s">
+      <c r="A15" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B15" s="6" t="s">
+      <c r="B15" s="7" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="6" t="s">
+      <c r="A16" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="B16" s="6" t="s">
+      <c r="B16" s="7" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="7" t="s">
+      <c r="A17" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="B17" s="6" t="s">
+      <c r="B17" s="7" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="8" t="s">
+      <c r="A19" s="9" t="s">
         <v>18</v>
       </c>
     </row>
@@ -1225,226 +1229,226 @@
   <dimension ref="A1:F20"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="58"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="58"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="9" t="s">
+      <c r="A2" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="B2" s="9"/>
-      <c r="C2" s="9"/>
-      <c r="D2" s="9"/>
-      <c r="E2" s="9"/>
-      <c r="F2" s="9"/>
+      <c r="B2" s="10"/>
+      <c r="C2" s="10"/>
+      <c r="D2" s="10"/>
+      <c r="E2" s="10"/>
+      <c r="F2" s="10"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="10" t="s">
+      <c r="A4" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="B4" s="10" t="s">
+      <c r="B4" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="C4" s="10" t="s">
+      <c r="C4" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="D4" s="10" t="s">
+      <c r="D4" s="11" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="11" t="s">
+      <c r="A5" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="B5" s="12" t="n">
+      <c r="B5" s="13" t="n">
         <v>25000000</v>
       </c>
-      <c r="C5" s="13" t="s">
+      <c r="C5" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="D5" s="14" t="s">
+      <c r="D5" s="15" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="11" t="s">
+      <c r="A6" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="B6" s="15" t="n">
+      <c r="B6" s="16" t="n">
         <v>0.35</v>
       </c>
-      <c r="C6" s="13" t="s">
+      <c r="C6" s="14" t="s">
         <v>29</v>
       </c>
-      <c r="D6" s="14" t="s">
+      <c r="D6" s="15" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="11" t="s">
+      <c r="A7" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="B7" s="15" t="n">
+      <c r="B7" s="16" t="n">
         <v>0.55</v>
       </c>
-      <c r="C7" s="13" t="s">
+      <c r="C7" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="D7" s="14" t="s">
+      <c r="D7" s="15" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="11" t="s">
+      <c r="A8" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="B8" s="15" t="n">
+      <c r="B8" s="16" t="n">
         <v>0.5</v>
       </c>
-      <c r="C8" s="13" t="s">
+      <c r="C8" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="D8" s="14" t="s">
+      <c r="D8" s="15" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="11" t="s">
+      <c r="A9" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="B9" s="12" t="n">
+      <c r="B9" s="13" t="n">
         <v>11000000</v>
       </c>
-      <c r="C9" s="13" t="s">
+      <c r="C9" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="D9" s="14" t="s">
+      <c r="D9" s="15" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="11" t="s">
+      <c r="A10" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="B10" s="15" t="n">
+      <c r="B10" s="16" t="n">
         <v>0.04</v>
       </c>
-      <c r="C10" s="13" t="s">
+      <c r="C10" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="D10" s="14" t="s">
+      <c r="D10" s="15" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="11" t="s">
+      <c r="A11" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="B11" s="12" t="n">
+      <c r="B11" s="13" t="n">
         <v>9000</v>
       </c>
-      <c r="C11" s="13" t="s">
+      <c r="C11" s="14" t="s">
         <v>42</v>
       </c>
-      <c r="D11" s="14" t="s">
+      <c r="D11" s="15" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="11" t="s">
+      <c r="A12" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="B12" s="12" t="n">
+      <c r="B12" s="13" t="n">
         <v>32</v>
       </c>
-      <c r="C12" s="13" t="s">
+      <c r="C12" s="14" t="s">
         <v>45</v>
       </c>
-      <c r="D12" s="14" t="s">
+      <c r="D12" s="15" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="11" t="s">
+      <c r="A13" s="12" t="s">
         <v>47</v>
       </c>
-      <c r="B13" s="12" t="n">
+      <c r="B13" s="13" t="n">
         <v>4000000</v>
       </c>
-      <c r="C13" s="13" t="s">
+      <c r="C13" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="D13" s="14" t="s">
+      <c r="D13" s="15" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="11" t="s">
+      <c r="A14" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="B14" s="15" t="n">
+      <c r="B14" s="16" t="n">
         <v>0.2</v>
       </c>
-      <c r="C14" s="13" t="s">
+      <c r="C14" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="D14" s="14" t="s">
+      <c r="D14" s="15" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="11" t="s">
+      <c r="A15" s="12" t="s">
         <v>53</v>
       </c>
-      <c r="B15" s="12" t="n">
+      <c r="B15" s="13" t="n">
         <v>1200000</v>
       </c>
-      <c r="C15" s="13" t="s">
+      <c r="C15" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="D15" s="14" t="s">
+      <c r="D15" s="15" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="16" t="s">
+      <c r="A17" s="17" t="s">
         <v>55</v>
       </c>
-      <c r="B17" s="17" t="n">
+      <c r="B17" s="18" t="n">
         <f aca="false">B9*B10</f>
         <v>440000</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="16" t="s">
+      <c r="A18" s="17" t="s">
         <v>56</v>
       </c>
-      <c r="B18" s="17" t="n">
+      <c r="B18" s="18" t="n">
         <f aca="false">B11*B12</f>
         <v>288000</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="16" t="s">
+      <c r="A19" s="17" t="s">
         <v>57</v>
       </c>
-      <c r="B19" s="17" t="n">
+      <c r="B19" s="18" t="n">
         <f aca="false">B13*B14</f>
         <v>800000</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="16" t="s">
+      <c r="A20" s="17" t="s">
         <v>58</v>
       </c>
-      <c r="B20" s="17" t="n">
+      <c r="B20" s="18" t="n">
         <f aca="false">IF(B7&gt;0,B5*(0.01/B7)*B8*B6,0)</f>
         <v>79545.4545454545</v>
       </c>
@@ -1473,179 +1477,179 @@
   <dimension ref="A1:F13"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="32"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="50"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="32"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="50"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="9" t="s">
+      <c r="A2" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="B2" s="9"/>
-      <c r="C2" s="9"/>
-      <c r="D2" s="9"/>
-      <c r="E2" s="9"/>
-      <c r="F2" s="9"/>
+      <c r="B2" s="10"/>
+      <c r="C2" s="10"/>
+      <c r="D2" s="10"/>
+      <c r="E2" s="10"/>
+      <c r="F2" s="10"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="10" t="s">
+      <c r="A4" s="11" t="s">
         <v>61</v>
       </c>
-      <c r="B4" s="10" t="s">
+      <c r="B4" s="11" t="s">
         <v>62</v>
       </c>
-      <c r="C4" s="10" t="s">
+      <c r="C4" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="D4" s="10" t="s">
+      <c r="D4" s="11" t="s">
         <v>64</v>
       </c>
-      <c r="E4" s="10" t="s">
+      <c r="E4" s="11" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="11" t="s">
+      <c r="A5" s="12" t="s">
         <v>66</v>
       </c>
-      <c r="B5" s="18" t="n">
+      <c r="B5" s="19" t="n">
         <v>5</v>
       </c>
-      <c r="C5" s="13" t="s">
+      <c r="C5" s="14" t="s">
         <v>67</v>
       </c>
-      <c r="D5" s="19" t="n">
+      <c r="D5" s="20" t="n">
         <f aca="false">Baseline!B20*B5</f>
         <v>397727.272727273</v>
       </c>
-      <c r="E5" s="14" t="s">
+      <c r="E5" s="15" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="11" t="s">
+      <c r="A6" s="12" t="s">
         <v>69</v>
       </c>
-      <c r="B6" s="15" t="n">
+      <c r="B6" s="16" t="n">
         <v>0.1</v>
       </c>
-      <c r="C6" s="13" t="s">
+      <c r="C6" s="14" t="s">
         <v>70</v>
       </c>
-      <c r="D6" s="19" t="n">
+      <c r="D6" s="20" t="n">
         <f aca="false">Baseline!B17*B6</f>
         <v>44000</v>
       </c>
-      <c r="E6" s="14" t="s">
+      <c r="E6" s="15" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="11" t="s">
+      <c r="A7" s="12" t="s">
         <v>72</v>
       </c>
-      <c r="B7" s="15" t="n">
+      <c r="B7" s="16" t="n">
         <v>0.5</v>
       </c>
-      <c r="C7" s="13" t="s">
+      <c r="C7" s="14" t="s">
         <v>73</v>
       </c>
-      <c r="D7" s="19" t="n">
+      <c r="D7" s="20" t="n">
         <f aca="false">Baseline!B18*B7</f>
         <v>144000</v>
       </c>
-      <c r="E7" s="14" t="s">
+      <c r="E7" s="15" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="11" t="s">
+      <c r="A8" s="12" t="s">
         <v>75</v>
       </c>
-      <c r="B8" s="15" t="n">
+      <c r="B8" s="16" t="n">
         <v>0.1</v>
       </c>
-      <c r="C8" s="13" t="s">
+      <c r="C8" s="14" t="s">
         <v>76</v>
       </c>
-      <c r="D8" s="19" t="n">
+      <c r="D8" s="20" t="n">
         <f aca="false">Baseline!B19*B8</f>
         <v>80000</v>
       </c>
-      <c r="E8" s="14" t="s">
+      <c r="E8" s="15" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="11" t="s">
+      <c r="A9" s="12" t="s">
         <v>78</v>
       </c>
-      <c r="B9" s="15" t="n">
+      <c r="B9" s="16" t="n">
         <v>0.05</v>
       </c>
-      <c r="C9" s="13" t="s">
+      <c r="C9" s="14" t="s">
         <v>79</v>
       </c>
-      <c r="D9" s="19" t="n">
+      <c r="D9" s="20" t="n">
         <f aca="false">Baseline!B15*B9</f>
         <v>60000</v>
       </c>
-      <c r="E9" s="14" t="s">
+      <c r="E9" s="15" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="16" t="s">
+      <c r="A10" s="17" t="s">
         <v>81</v>
       </c>
-      <c r="D10" s="17" t="n">
+      <c r="D10" s="18" t="n">
         <f aca="false">SUM(D5:D9)</f>
         <v>725727.272727273</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="16" t="s">
+      <c r="B11" s="17" t="s">
         <v>82</v>
       </c>
-      <c r="C11" s="16" t="s">
+      <c r="C11" s="17" t="s">
         <v>83</v>
       </c>
-      <c r="D11" s="16" t="s">
+      <c r="D11" s="17" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="16" t="s">
+      <c r="A12" s="17" t="s">
         <v>85</v>
       </c>
-      <c r="B12" s="15" t="n">
+      <c r="B12" s="16" t="n">
         <v>0.4</v>
       </c>
-      <c r="C12" s="15" t="n">
+      <c r="C12" s="16" t="n">
         <v>0.8</v>
       </c>
-      <c r="D12" s="15" t="n">
+      <c r="D12" s="16" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="13" t="s">
+      <c r="A13" s="14" t="s">
         <v>86</v>
       </c>
-      <c r="B13" s="14" t="s">
+      <c r="B13" s="15" t="s">
         <v>87</v>
       </c>
-      <c r="C13" s="14"/>
-      <c r="D13" s="14"/>
-      <c r="E13" s="14"/>
+      <c r="C13" s="15"/>
+      <c r="D13" s="15"/>
+      <c r="E13" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1671,233 +1675,233 @@
   <dimension ref="A1:F14"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="3" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="3" style="1" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="52"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="9" t="s">
+      <c r="A2" s="10" t="s">
         <v>89</v>
       </c>
-      <c r="B2" s="9"/>
-      <c r="C2" s="9"/>
-      <c r="D2" s="9"/>
-      <c r="E2" s="9"/>
-      <c r="F2" s="9"/>
+      <c r="B2" s="10"/>
+      <c r="C2" s="10"/>
+      <c r="D2" s="10"/>
+      <c r="E2" s="10"/>
+      <c r="F2" s="10"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="10" t="s">
+      <c r="A4" s="11" t="s">
         <v>90</v>
       </c>
-      <c r="B4" s="10" t="s">
+      <c r="B4" s="11" t="s">
         <v>91</v>
       </c>
-      <c r="C4" s="10" t="s">
+      <c r="C4" s="11" t="s">
         <v>82</v>
       </c>
-      <c r="D4" s="10" t="s">
+      <c r="D4" s="11" t="s">
         <v>83</v>
       </c>
-      <c r="E4" s="10" t="s">
+      <c r="E4" s="11" t="s">
         <v>84</v>
       </c>
-      <c r="F4" s="10" t="s">
+      <c r="F4" s="11" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="11" t="s">
+      <c r="A5" s="12" t="s">
         <v>92</v>
       </c>
-      <c r="B5" s="12" t="n">
+      <c r="B5" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="C5" s="12" t="n">
+      <c r="C5" s="13" t="n">
         <v>90000</v>
       </c>
-      <c r="D5" s="12" t="n">
+      <c r="D5" s="13" t="n">
         <v>90000</v>
       </c>
-      <c r="E5" s="12" t="n">
+      <c r="E5" s="13" t="n">
         <v>90000</v>
       </c>
-      <c r="F5" s="14" t="s">
+      <c r="F5" s="15" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="11" t="s">
+      <c r="A6" s="12" t="s">
         <v>94</v>
       </c>
-      <c r="B6" s="12" t="n">
+      <c r="B6" s="13" t="n">
         <v>250000</v>
       </c>
-      <c r="C6" s="12" t="n">
+      <c r="C6" s="13" t="n">
         <v>30000</v>
       </c>
-      <c r="D6" s="12" t="n">
+      <c r="D6" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="E6" s="12" t="n">
+      <c r="E6" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="F6" s="14" t="s">
+      <c r="F6" s="15" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="11" t="s">
+      <c r="A7" s="12" t="s">
         <v>96</v>
       </c>
-      <c r="B7" s="12" t="n">
+      <c r="B7" s="13" t="n">
         <v>80000</v>
       </c>
-      <c r="C7" s="12" t="n">
+      <c r="C7" s="13" t="n">
         <v>10000</v>
       </c>
-      <c r="D7" s="12" t="n">
+      <c r="D7" s="13" t="n">
         <v>10000</v>
       </c>
-      <c r="E7" s="12" t="n">
+      <c r="E7" s="13" t="n">
         <v>10000</v>
       </c>
-      <c r="F7" s="14" t="s">
+      <c r="F7" s="15" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="11" t="s">
+      <c r="A8" s="12" t="s">
         <v>98</v>
       </c>
-      <c r="B8" s="12" t="n">
+      <c r="B8" s="13" t="n">
         <v>60000</v>
       </c>
-      <c r="C8" s="12" t="n">
+      <c r="C8" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="D8" s="12" t="n">
+      <c r="D8" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="E8" s="12" t="n">
+      <c r="E8" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="F8" s="14" t="s">
+      <c r="F8" s="15" t="s">
         <v>99</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="11" t="s">
+      <c r="A9" s="12" t="s">
         <v>100</v>
       </c>
-      <c r="B9" s="12" t="n">
+      <c r="B9" s="13" t="n">
         <v>150000</v>
       </c>
-      <c r="C9" s="12" t="n">
+      <c r="C9" s="13" t="n">
         <v>80000</v>
       </c>
-      <c r="D9" s="12" t="n">
+      <c r="D9" s="13" t="n">
         <v>40000</v>
       </c>
-      <c r="E9" s="12" t="n">
+      <c r="E9" s="13" t="n">
         <v>40000</v>
       </c>
-      <c r="F9" s="14" t="s">
+      <c r="F9" s="15" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="11" t="s">
+      <c r="A10" s="12" t="s">
         <v>102</v>
       </c>
-      <c r="B10" s="12" t="n">
+      <c r="B10" s="13" t="n">
         <v>30000</v>
       </c>
-      <c r="C10" s="12" t="n">
+      <c r="C10" s="13" t="n">
         <v>10000</v>
       </c>
-      <c r="D10" s="12" t="n">
+      <c r="D10" s="13" t="n">
         <v>5000</v>
       </c>
-      <c r="E10" s="12" t="n">
+      <c r="E10" s="13" t="n">
         <v>5000</v>
       </c>
-      <c r="F10" s="14" t="s">
+      <c r="F10" s="15" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="11" t="s">
+      <c r="A11" s="12" t="s">
         <v>104</v>
       </c>
-      <c r="B11" s="12" t="n">
+      <c r="B11" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="C11" s="12" t="n">
+      <c r="C11" s="13" t="n">
         <v>25000</v>
       </c>
-      <c r="D11" s="12" t="n">
+      <c r="D11" s="13" t="n">
         <v>25000</v>
       </c>
-      <c r="E11" s="12" t="n">
+      <c r="E11" s="13" t="n">
         <v>25000</v>
       </c>
-      <c r="F11" s="14" t="s">
+      <c r="F11" s="15" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="16" t="s">
+      <c r="A12" s="17" t="s">
         <v>106</v>
       </c>
-      <c r="B12" s="20" t="n">
+      <c r="B12" s="21" t="n">
         <f aca="false">SUM(B5:B11)*$B$13</f>
         <v>85500</v>
       </c>
-      <c r="C12" s="20" t="n">
+      <c r="C12" s="21" t="n">
         <f aca="false">SUM(C5:C11)*$B$13</f>
         <v>36750</v>
       </c>
-      <c r="D12" s="20" t="n">
+      <c r="D12" s="21" t="n">
         <f aca="false">SUM(D5:D11)*$B$13</f>
         <v>25500</v>
       </c>
-      <c r="E12" s="20" t="n">
+      <c r="E12" s="21" t="n">
         <f aca="false">SUM(E5:E11)*$B$13</f>
         <v>25500</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="11" t="s">
+      <c r="A13" s="12" t="s">
         <v>107</v>
       </c>
-      <c r="B13" s="15" t="n">
+      <c r="B13" s="16" t="n">
         <v>0.15</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="16" t="s">
+      <c r="A14" s="17" t="s">
         <v>108</v>
       </c>
-      <c r="B14" s="17" t="n">
+      <c r="B14" s="18" t="n">
         <f aca="false">SUM(B5:B12)</f>
         <v>655500</v>
       </c>
-      <c r="C14" s="17" t="n">
+      <c r="C14" s="18" t="n">
         <f aca="false">SUM(C5:C12)</f>
         <v>281750</v>
       </c>
-      <c r="D14" s="17" t="n">
+      <c r="D14" s="18" t="n">
         <f aca="false">SUM(D5:D12)</f>
         <v>195500</v>
       </c>
-      <c r="E14" s="17" t="n">
+      <c r="E14" s="18" t="n">
         <f aca="false">SUM(E5:E12)</f>
         <v>195500</v>
       </c>
@@ -1925,177 +1929,177 @@
   <dimension ref="A1:F16"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="2" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="2" style="1" width="15"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="9" t="s">
+      <c r="A2" s="10" t="s">
         <v>110</v>
       </c>
-      <c r="B2" s="9"/>
-      <c r="C2" s="9"/>
-      <c r="D2" s="9"/>
-      <c r="E2" s="9"/>
-      <c r="F2" s="9"/>
+      <c r="B2" s="10"/>
+      <c r="C2" s="10"/>
+      <c r="D2" s="10"/>
+      <c r="E2" s="10"/>
+      <c r="F2" s="10"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="10"/>
-      <c r="B4" s="10" t="s">
+      <c r="A4" s="11"/>
+      <c r="B4" s="11" t="s">
         <v>111</v>
       </c>
-      <c r="C4" s="10" t="s">
+      <c r="C4" s="11" t="s">
         <v>82</v>
       </c>
-      <c r="D4" s="10" t="s">
+      <c r="D4" s="11" t="s">
         <v>83</v>
       </c>
-      <c r="E4" s="10" t="s">
+      <c r="E4" s="11" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="11" t="s">
+      <c r="A5" s="12" t="s">
         <v>112</v>
       </c>
-      <c r="B5" s="20" t="n">
+      <c r="B5" s="21" t="n">
         <v>0</v>
       </c>
-      <c r="C5" s="19" t="n">
+      <c r="C5" s="20" t="n">
         <f aca="false">Benefits!$D$10*Benefits!B12</f>
         <v>290290.909090909</v>
       </c>
-      <c r="D5" s="19" t="n">
+      <c r="D5" s="20" t="n">
         <f aca="false">Benefits!$D$10*Benefits!C12</f>
         <v>580581.818181818</v>
       </c>
-      <c r="E5" s="19" t="n">
+      <c r="E5" s="20" t="n">
         <f aca="false">Benefits!$D$10*Benefits!D12</f>
         <v>725727.272727273</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="11" t="s">
+      <c r="A6" s="12" t="s">
         <v>113</v>
       </c>
-      <c r="B6" s="19" t="n">
+      <c r="B6" s="20" t="n">
         <f aca="false">-Costs!B14</f>
         <v>-655500</v>
       </c>
-      <c r="C6" s="19" t="n">
+      <c r="C6" s="20" t="n">
         <f aca="false">-Costs!C14</f>
         <v>-281750</v>
       </c>
-      <c r="D6" s="19" t="n">
+      <c r="D6" s="20" t="n">
         <f aca="false">-Costs!D14</f>
         <v>-195500</v>
       </c>
-      <c r="E6" s="19" t="n">
+      <c r="E6" s="20" t="n">
         <f aca="false">-Costs!E14</f>
         <v>-195500</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="16" t="s">
+      <c r="A7" s="17" t="s">
         <v>114</v>
       </c>
-      <c r="B7" s="21" t="n">
+      <c r="B7" s="22" t="n">
         <f aca="false">B5+B6</f>
         <v>-655500</v>
       </c>
-      <c r="C7" s="21" t="n">
+      <c r="C7" s="22" t="n">
         <f aca="false">C5+C6</f>
         <v>8540.90909090912</v>
       </c>
-      <c r="D7" s="21" t="n">
+      <c r="D7" s="22" t="n">
         <f aca="false">D5+D6</f>
         <v>385081.818181818</v>
       </c>
-      <c r="E7" s="21" t="n">
+      <c r="E7" s="22" t="n">
         <f aca="false">E5+E6</f>
         <v>530227.272727273</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="16" t="s">
+      <c r="A8" s="17" t="s">
         <v>115</v>
       </c>
-      <c r="B8" s="17" t="n">
+      <c r="B8" s="18" t="n">
         <f aca="false">B7</f>
         <v>-655500</v>
       </c>
-      <c r="C8" s="17" t="n">
+      <c r="C8" s="18" t="n">
         <f aca="false">B8+C7</f>
         <v>-646959.090909091</v>
       </c>
-      <c r="D8" s="17" t="n">
+      <c r="D8" s="18" t="n">
         <f aca="false">C8+D7</f>
         <v>-261877.272727273</v>
       </c>
-      <c r="E8" s="17" t="n">
+      <c r="E8" s="18" t="n">
         <f aca="false">D8+E7</f>
         <v>268350</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="16" t="s">
+      <c r="A10" s="17" t="s">
         <v>116</v>
       </c>
-      <c r="B10" s="21" t="n">
+      <c r="B10" s="22" t="n">
         <f aca="false">SUM(C5:E5)</f>
         <v>1596600</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="16" t="s">
+      <c r="A11" s="17" t="s">
         <v>117</v>
       </c>
-      <c r="B11" s="21" t="n">
+      <c r="B11" s="22" t="n">
         <f aca="false">-SUM(B6:E6)</f>
         <v>1328250</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="16" t="s">
+      <c r="A12" s="17" t="s">
         <v>118</v>
       </c>
-      <c r="B12" s="17" t="n">
+      <c r="B12" s="18" t="n">
         <f aca="false">B10-B11</f>
         <v>268350</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="16" t="s">
+      <c r="A13" s="17" t="s">
         <v>119</v>
       </c>
-      <c r="B13" s="22" t="n">
+      <c r="B13" s="23" t="n">
         <f aca="false">IF(B11&gt;0,B12/B11,0)</f>
         <v>0.202032749858837</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="16" t="s">
+      <c r="A14" s="17" t="s">
         <v>120</v>
       </c>
-      <c r="B14" s="23" t="str">
+      <c r="B14" s="24" t="str">
         <f aca="false">IF(C8&gt;=0,"Year 1",IF(D8&gt;=0,"Year 2",IF(E8&gt;=0,"Year 3","After year 3")))</f>
         <v>Year 3</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="16" t="s">
+      <c r="A16" s="17" t="s">
         <v>121</v>
       </c>
-      <c r="B16" s="19" t="n">
+      <c r="B16" s="20" t="n">
         <f aca="false">Benefits!D10</f>
         <v>725727.272727273</v>
       </c>
-      <c r="C16" s="13" t="s">
+      <c r="C16" s="14" t="s">
         <v>122</v>
       </c>
     </row>
@@ -2127,132 +2131,132 @@
   <dimension ref="A1:F10"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="36"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="20"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>123</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="9" t="s">
+      <c r="A2" s="10" t="s">
         <v>124</v>
       </c>
-      <c r="B2" s="9"/>
-      <c r="C2" s="9"/>
-      <c r="D2" s="9"/>
-      <c r="E2" s="9"/>
-      <c r="F2" s="9"/>
+      <c r="B2" s="10"/>
+      <c r="C2" s="10"/>
+      <c r="D2" s="10"/>
+      <c r="E2" s="10"/>
+      <c r="F2" s="10"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="10" t="s">
+      <c r="A4" s="11" t="s">
         <v>125</v>
       </c>
-      <c r="B4" s="10" t="s">
+      <c r="B4" s="11" t="s">
         <v>126</v>
       </c>
-      <c r="C4" s="10" t="s">
+      <c r="C4" s="11" t="s">
         <v>127</v>
       </c>
-      <c r="D4" s="10" t="s">
+      <c r="D4" s="11" t="s">
         <v>128</v>
       </c>
-      <c r="E4" s="10" t="s">
+      <c r="E4" s="11" t="s">
         <v>129</v>
       </c>
-      <c r="F4" s="10" t="s">
+      <c r="F4" s="11" t="s">
         <v>130</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="24" t="s">
+      <c r="A5" s="25" t="s">
         <v>131</v>
       </c>
-      <c r="B5" s="24" t="s">
+      <c r="B5" s="25" t="s">
         <v>132</v>
       </c>
-      <c r="C5" s="24" t="s">
+      <c r="C5" s="25" t="s">
         <v>133</v>
       </c>
-      <c r="D5" s="24" t="s">
+      <c r="D5" s="25" t="s">
         <v>134</v>
       </c>
-      <c r="E5" s="24" t="s">
+      <c r="E5" s="25" t="s">
         <v>135</v>
       </c>
-      <c r="F5" s="24" t="s">
+      <c r="F5" s="25" t="s">
         <v>136</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="24" t="s">
+      <c r="A6" s="25" t="s">
         <v>137</v>
       </c>
-      <c r="B6" s="24" t="s">
+      <c r="B6" s="25" t="s">
         <v>138</v>
       </c>
-      <c r="C6" s="24" t="s">
+      <c r="C6" s="25" t="s">
         <v>139</v>
       </c>
-      <c r="D6" s="24" t="s">
+      <c r="D6" s="25" t="s">
         <v>140</v>
       </c>
-      <c r="E6" s="24" t="s">
+      <c r="E6" s="25" t="s">
         <v>141</v>
       </c>
-      <c r="F6" s="24" t="s">
+      <c r="F6" s="25" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="24" t="s">
+      <c r="A7" s="25" t="s">
         <v>143</v>
       </c>
-      <c r="B7" s="24" t="s">
+      <c r="B7" s="25" t="s">
         <v>144</v>
       </c>
-      <c r="C7" s="24" t="s">
-        <v>133</v>
-      </c>
-      <c r="D7" s="24" t="s">
+      <c r="C7" s="25" t="s">
         <v>145</v>
       </c>
-      <c r="E7" s="24" t="s">
+      <c r="D7" s="25" t="s">
         <v>146</v>
       </c>
-      <c r="F7" s="24" t="s">
+      <c r="E7" s="25" t="s">
         <v>147</v>
       </c>
+      <c r="F7" s="25" t="s">
+        <v>142</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="25"/>
-      <c r="B8" s="25"/>
-      <c r="C8" s="25"/>
-      <c r="D8" s="25"/>
-      <c r="E8" s="25"/>
-      <c r="F8" s="25"/>
+      <c r="A8" s="26"/>
+      <c r="B8" s="26"/>
+      <c r="C8" s="26"/>
+      <c r="D8" s="26"/>
+      <c r="E8" s="26"/>
+      <c r="F8" s="26"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="25"/>
-      <c r="B9" s="25"/>
-      <c r="C9" s="25"/>
-      <c r="D9" s="25"/>
-      <c r="E9" s="25"/>
-      <c r="F9" s="25"/>
+      <c r="A9" s="26"/>
+      <c r="B9" s="26"/>
+      <c r="C9" s="26"/>
+      <c r="D9" s="26"/>
+      <c r="E9" s="26"/>
+      <c r="F9" s="26"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="25"/>
-      <c r="B10" s="25"/>
-      <c r="C10" s="25"/>
-      <c r="D10" s="25"/>
-      <c r="E10" s="25"/>
-      <c r="F10" s="25"/>
+      <c r="A10" s="26"/>
+      <c r="B10" s="26"/>
+      <c r="C10" s="26"/>
+      <c r="D10" s="26"/>
+      <c r="E10" s="26"/>
+      <c r="F10" s="26"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Revert "Business case: commit to every site, no phased funding; 1% question; intangibles wording; template rollout sheet"
This reverts commit c25233c929dbf0f9470f1058ddbe899a467ccb1a.
</commit_message>
<xml_diff>
--- a/public/downloads/shopfloor-matters-business-case-template.xlsx
+++ b/public/downloads/shopfloor-matters-business-case-template.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Benefits" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="Costs" sheetId="4" state="visible" r:id="rId6"/>
     <sheet name="Cash flow" sheetId="5" state="visible" r:id="rId7"/>
-    <sheet name="Rollout" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="Phasing" sheetId="6" state="visible" r:id="rId8"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -64,7 +64,7 @@
     <t xml:space="preserve">3. Realistic costs and timeline, including your own people, not just licences and services (Costs).</t>
   </si>
   <si>
-    <t xml:space="preserve">4. How the risk is managed: a clear rollout plan across every site, with milestones and measures (Rollout).</t>
+    <t xml:space="preserve">4. How the risk is managed: phases, measures and decision points (Phasing).</t>
   </si>
   <si>
     <t xml:space="preserve">How to use it:</t>
@@ -73,7 +73,7 @@
     <t xml:space="preserve">Fill in Baseline with numbers finance will recognise. Set deliberately modest improvements on Benefits. Fill in every cost line, then read Cash flow.</t>
   </si>
   <si>
-    <t xml:space="preserve">Make the case for every site as one programme: licences for all your sites, a template built on the first, and a clear plan for the rest.</t>
+    <t xml:space="preserve">Keep the first phase small: one line or one area. Let its results fund the next phase.</t>
   </si>
   <si>
     <t xml:space="preserve">The example values describe a fictional mid-size site so you can see how it works. They are not a forecast. Replace them all.</t>
@@ -418,13 +418,13 @@
     <t xml:space="preserve">Every year you wait, this is what stays on the table.</t>
   </si>
   <si>
-    <t xml:space="preserve">Rollout: how the risk is managed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The section boards read most closely. The programme covers every site. Each stage has a scope, a measure and a milestone, so progress is visible all the way.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Stage</t>
+    <t xml:space="preserve">Phasing: how the risk is managed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The section boards read most closely. Each phase has a scope, a measure and a decision point. The next phase only starts when the measure says so.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phase</t>
   </si>
   <si>
     <t xml:space="preserve">Scope</t>
@@ -436,61 +436,61 @@
     <t xml:space="preserve">Success measure</t>
   </si>
   <si>
-    <t xml:space="preserve">Milestone</t>
+    <t xml:space="preserve">Decision point</t>
   </si>
   <si>
     <t xml:space="preserve">Owner</t>
   </si>
   <si>
-    <t xml:space="preserve">1. First site</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The whole site, starting with production and quality</t>
+    <t xml:space="preserve">1. Pilot</t>
+  </si>
+  <si>
+    <t xml:space="preserve">One line, production and quality</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4 to 6 months</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OEE up 3 points against baseline; scrap down 10%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Steering group review at month 6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Operations director</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2. Site</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Remaining lines on the site</t>
   </si>
   <si>
     <t xml:space="preserve">6 to 9 months</t>
   </si>
   <si>
-    <t xml:space="preserve">OEE up 3 points against baseline; scrap down 10%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">First site live on every shift</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Operations director</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2. Template</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Standard processes, master data rules, KPIs and screens from the first site</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2 to 3 months</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Template signed off by the centre of excellence</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Template ready for the next site</t>
+    <t xml:space="preserve">Benefits on Benefits sheet reached at 80% ramp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Before committing to site 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Site lead</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3. Template</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Second site from the same template</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Go-live on time with under 10% local change</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Before wider roll-out</t>
   </si>
   <si>
     <t xml:space="preserve">Programme lead</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3. Remaining sites</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Every other site, from the same template</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4 to 6 months per site</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Go-live on time with under 10% local change; benefits on Benefits sheet reached</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Each site live on every shift</t>
   </si>
 </sst>
 </file>
@@ -658,112 +658,108 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="26">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="166" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="167" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1034,166 +1030,166 @@
   <dimension ref="A1:H19"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="2" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="2" style="0" width="14"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
-      <c r="G3" s="3"/>
-      <c r="H3" s="3"/>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="4"/>
-      <c r="C4" s="4"/>
-      <c r="D4" s="4"/>
-      <c r="E4" s="4"/>
-      <c r="F4" s="4"/>
-      <c r="G4" s="4"/>
-      <c r="H4" s="4"/>
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
     </row>
     <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="4"/>
-      <c r="C5" s="4"/>
-      <c r="D5" s="4"/>
-      <c r="E5" s="4"/>
-      <c r="F5" s="4"/>
-      <c r="G5" s="4"/>
-      <c r="H5" s="4"/>
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3"/>
+      <c r="H5" s="3"/>
     </row>
     <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="4"/>
-      <c r="C6" s="4"/>
-      <c r="D6" s="4"/>
-      <c r="E6" s="4"/>
-      <c r="F6" s="4"/>
-      <c r="G6" s="4"/>
-      <c r="H6" s="4"/>
-    </row>
-    <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="s">
+      <c r="B6" s="3"/>
+      <c r="C6" s="3"/>
+      <c r="D6" s="3"/>
+      <c r="E6" s="3"/>
+      <c r="F6" s="3"/>
+      <c r="G6" s="3"/>
+      <c r="H6" s="3"/>
+    </row>
+    <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="4"/>
-      <c r="C7" s="4"/>
-      <c r="D7" s="4"/>
-      <c r="E7" s="4"/>
-      <c r="F7" s="4"/>
-      <c r="G7" s="4"/>
-      <c r="H7" s="4"/>
+      <c r="B7" s="3"/>
+      <c r="C7" s="3"/>
+      <c r="D7" s="3"/>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
+      <c r="G7" s="3"/>
+      <c r="H7" s="3"/>
     </row>
     <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3" t="s">
+      <c r="A8" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="3"/>
-      <c r="C8" s="3"/>
-      <c r="D8" s="3"/>
-      <c r="E8" s="3"/>
-      <c r="F8" s="3"/>
-      <c r="G8" s="3"/>
-      <c r="H8" s="3"/>
+      <c r="B8" s="2"/>
+      <c r="C8" s="2"/>
+      <c r="D8" s="2"/>
+      <c r="E8" s="2"/>
+      <c r="F8" s="2"/>
+      <c r="G8" s="2"/>
+      <c r="H8" s="2"/>
     </row>
     <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4" t="s">
+      <c r="A9" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="4"/>
-      <c r="C9" s="4"/>
-      <c r="D9" s="4"/>
-      <c r="E9" s="4"/>
-      <c r="F9" s="4"/>
-      <c r="G9" s="4"/>
-      <c r="H9" s="4"/>
-    </row>
-    <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4" t="s">
+      <c r="B9" s="3"/>
+      <c r="C9" s="3"/>
+      <c r="D9" s="3"/>
+      <c r="E9" s="3"/>
+      <c r="F9" s="3"/>
+      <c r="G9" s="3"/>
+      <c r="H9" s="3"/>
+    </row>
+    <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="4"/>
-      <c r="C10" s="4"/>
-      <c r="D10" s="4"/>
-      <c r="E10" s="4"/>
-      <c r="F10" s="4"/>
-      <c r="G10" s="4"/>
-      <c r="H10" s="4"/>
+      <c r="B10" s="3"/>
+      <c r="C10" s="3"/>
+      <c r="D10" s="3"/>
+      <c r="E10" s="3"/>
+      <c r="F10" s="3"/>
+      <c r="G10" s="3"/>
+      <c r="H10" s="3"/>
     </row>
     <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="s">
+      <c r="A11" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B11" s="4"/>
-      <c r="C11" s="4"/>
-      <c r="D11" s="4"/>
-      <c r="E11" s="4"/>
-      <c r="F11" s="4"/>
-      <c r="G11" s="4"/>
-      <c r="H11" s="4"/>
+      <c r="B11" s="3"/>
+      <c r="C11" s="3"/>
+      <c r="D11" s="3"/>
+      <c r="E11" s="3"/>
+      <c r="F11" s="3"/>
+      <c r="G11" s="3"/>
+      <c r="H11" s="3"/>
     </row>
     <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="4" t="s">
+      <c r="A12" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B12" s="4"/>
-      <c r="C12" s="4"/>
-      <c r="D12" s="4"/>
-      <c r="E12" s="4"/>
-      <c r="F12" s="4"/>
-      <c r="G12" s="4"/>
-      <c r="H12" s="4"/>
+      <c r="B12" s="3"/>
+      <c r="C12" s="3"/>
+      <c r="D12" s="3"/>
+      <c r="E12" s="3"/>
+      <c r="F12" s="3"/>
+      <c r="G12" s="3"/>
+      <c r="H12" s="3"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="5" t="s">
+      <c r="A14" s="4" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="6" t="s">
+      <c r="A15" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B15" s="7" t="s">
+      <c r="B15" s="6" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="7" t="s">
+      <c r="A16" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="B16" s="7" t="s">
+      <c r="B16" s="6" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="8" t="s">
+      <c r="A17" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="B17" s="7" t="s">
+      <c r="B17" s="6" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="9" t="s">
+      <c r="A19" s="8" t="s">
         <v>18</v>
       </c>
     </row>
@@ -1229,226 +1225,226 @@
   <dimension ref="A1:F20"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="58"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="58"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="10" t="s">
+      <c r="A2" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="B2" s="10"/>
-      <c r="C2" s="10"/>
-      <c r="D2" s="10"/>
-      <c r="E2" s="10"/>
-      <c r="F2" s="10"/>
+      <c r="B2" s="9"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="11" t="s">
+      <c r="A4" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="B4" s="11" t="s">
+      <c r="B4" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="C4" s="11" t="s">
+      <c r="C4" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="D4" s="11" t="s">
+      <c r="D4" s="10" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="12" t="s">
+      <c r="A5" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="B5" s="13" t="n">
+      <c r="B5" s="12" t="n">
         <v>25000000</v>
       </c>
-      <c r="C5" s="14" t="s">
+      <c r="C5" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="D5" s="15" t="s">
+      <c r="D5" s="14" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="12" t="s">
+      <c r="A6" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="B6" s="16" t="n">
+      <c r="B6" s="15" t="n">
         <v>0.35</v>
       </c>
-      <c r="C6" s="14" t="s">
+      <c r="C6" s="13" t="s">
         <v>29</v>
       </c>
-      <c r="D6" s="15" t="s">
+      <c r="D6" s="14" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="12" t="s">
+      <c r="A7" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="B7" s="16" t="n">
+      <c r="B7" s="15" t="n">
         <v>0.55</v>
       </c>
-      <c r="C7" s="14" t="s">
+      <c r="C7" s="13" t="s">
         <v>32</v>
       </c>
-      <c r="D7" s="15" t="s">
+      <c r="D7" s="14" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="12" t="s">
+      <c r="A8" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="B8" s="16" t="n">
+      <c r="B8" s="15" t="n">
         <v>0.5</v>
       </c>
-      <c r="C8" s="14" t="s">
+      <c r="C8" s="13" t="s">
         <v>32</v>
       </c>
-      <c r="D8" s="15" t="s">
+      <c r="D8" s="14" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="12" t="s">
+      <c r="A9" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="B9" s="13" t="n">
+      <c r="B9" s="12" t="n">
         <v>11000000</v>
       </c>
-      <c r="C9" s="14" t="s">
+      <c r="C9" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="D9" s="15" t="s">
+      <c r="D9" s="14" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="12" t="s">
+      <c r="A10" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="B10" s="16" t="n">
+      <c r="B10" s="15" t="n">
         <v>0.04</v>
       </c>
-      <c r="C10" s="14" t="s">
+      <c r="C10" s="13" t="s">
         <v>39</v>
       </c>
-      <c r="D10" s="15" t="s">
+      <c r="D10" s="14" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="12" t="s">
+      <c r="A11" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="B11" s="13" t="n">
+      <c r="B11" s="12" t="n">
         <v>9000</v>
       </c>
-      <c r="C11" s="14" t="s">
+      <c r="C11" s="13" t="s">
         <v>42</v>
       </c>
-      <c r="D11" s="15" t="s">
+      <c r="D11" s="14" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="12" t="s">
+      <c r="A12" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="B12" s="13" t="n">
+      <c r="B12" s="12" t="n">
         <v>32</v>
       </c>
-      <c r="C12" s="14" t="s">
+      <c r="C12" s="13" t="s">
         <v>45</v>
       </c>
-      <c r="D12" s="15" t="s">
+      <c r="D12" s="14" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="12" t="s">
+      <c r="A13" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="B13" s="13" t="n">
+      <c r="B13" s="12" t="n">
         <v>4000000</v>
       </c>
-      <c r="C13" s="14" t="s">
+      <c r="C13" s="13" t="s">
         <v>48</v>
       </c>
-      <c r="D13" s="15" t="s">
+      <c r="D13" s="14" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="12" t="s">
+      <c r="A14" s="11" t="s">
         <v>50</v>
       </c>
-      <c r="B14" s="16" t="n">
+      <c r="B14" s="15" t="n">
         <v>0.2</v>
       </c>
-      <c r="C14" s="14" t="s">
+      <c r="C14" s="13" t="s">
         <v>51</v>
       </c>
-      <c r="D14" s="15" t="s">
+      <c r="D14" s="14" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="12" t="s">
+      <c r="A15" s="11" t="s">
         <v>53</v>
       </c>
-      <c r="B15" s="13" t="n">
+      <c r="B15" s="12" t="n">
         <v>1200000</v>
       </c>
-      <c r="C15" s="14" t="s">
+      <c r="C15" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="D15" s="15" t="s">
+      <c r="D15" s="14" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="17" t="s">
+      <c r="A17" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="B17" s="18" t="n">
+      <c r="B17" s="17" t="n">
         <f aca="false">B9*B10</f>
         <v>440000</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="17" t="s">
+      <c r="A18" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="B18" s="18" t="n">
+      <c r="B18" s="17" t="n">
         <f aca="false">B11*B12</f>
         <v>288000</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="17" t="s">
+      <c r="A19" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="B19" s="18" t="n">
+      <c r="B19" s="17" t="n">
         <f aca="false">B13*B14</f>
         <v>800000</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="17" t="s">
+      <c r="A20" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="B20" s="18" t="n">
+      <c r="B20" s="17" t="n">
         <f aca="false">IF(B7&gt;0,B5*(0.01/B7)*B8*B6,0)</f>
         <v>79545.4545454545</v>
       </c>
@@ -1477,179 +1473,179 @@
   <dimension ref="A1:F13"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="32"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="50"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="32"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="50"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="10" t="s">
+      <c r="A2" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="B2" s="10"/>
-      <c r="C2" s="10"/>
-      <c r="D2" s="10"/>
-      <c r="E2" s="10"/>
-      <c r="F2" s="10"/>
+      <c r="B2" s="9"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="11" t="s">
+      <c r="A4" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="B4" s="11" t="s">
+      <c r="B4" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="C4" s="11" t="s">
+      <c r="C4" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="D4" s="11" t="s">
+      <c r="D4" s="10" t="s">
         <v>64</v>
       </c>
-      <c r="E4" s="11" t="s">
+      <c r="E4" s="10" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="12" t="s">
+      <c r="A5" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="B5" s="19" t="n">
+      <c r="B5" s="18" t="n">
         <v>5</v>
       </c>
-      <c r="C5" s="14" t="s">
+      <c r="C5" s="13" t="s">
         <v>67</v>
       </c>
-      <c r="D5" s="20" t="n">
+      <c r="D5" s="19" t="n">
         <f aca="false">Baseline!B20*B5</f>
         <v>397727.272727273</v>
       </c>
-      <c r="E5" s="15" t="s">
+      <c r="E5" s="14" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="12" t="s">
+      <c r="A6" s="11" t="s">
         <v>69</v>
       </c>
-      <c r="B6" s="16" t="n">
+      <c r="B6" s="15" t="n">
         <v>0.1</v>
       </c>
-      <c r="C6" s="14" t="s">
+      <c r="C6" s="13" t="s">
         <v>70</v>
       </c>
-      <c r="D6" s="20" t="n">
+      <c r="D6" s="19" t="n">
         <f aca="false">Baseline!B17*B6</f>
         <v>44000</v>
       </c>
-      <c r="E6" s="15" t="s">
+      <c r="E6" s="14" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="12" t="s">
+      <c r="A7" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="B7" s="16" t="n">
+      <c r="B7" s="15" t="n">
         <v>0.5</v>
       </c>
-      <c r="C7" s="14" t="s">
+      <c r="C7" s="13" t="s">
         <v>73</v>
       </c>
-      <c r="D7" s="20" t="n">
+      <c r="D7" s="19" t="n">
         <f aca="false">Baseline!B18*B7</f>
         <v>144000</v>
       </c>
-      <c r="E7" s="15" t="s">
+      <c r="E7" s="14" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="12" t="s">
+      <c r="A8" s="11" t="s">
         <v>75</v>
       </c>
-      <c r="B8" s="16" t="n">
+      <c r="B8" s="15" t="n">
         <v>0.1</v>
       </c>
-      <c r="C8" s="14" t="s">
+      <c r="C8" s="13" t="s">
         <v>76</v>
       </c>
-      <c r="D8" s="20" t="n">
+      <c r="D8" s="19" t="n">
         <f aca="false">Baseline!B19*B8</f>
         <v>80000</v>
       </c>
-      <c r="E8" s="15" t="s">
+      <c r="E8" s="14" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="12" t="s">
+      <c r="A9" s="11" t="s">
         <v>78</v>
       </c>
-      <c r="B9" s="16" t="n">
+      <c r="B9" s="15" t="n">
         <v>0.05</v>
       </c>
-      <c r="C9" s="14" t="s">
+      <c r="C9" s="13" t="s">
         <v>79</v>
       </c>
-      <c r="D9" s="20" t="n">
+      <c r="D9" s="19" t="n">
         <f aca="false">Baseline!B15*B9</f>
         <v>60000</v>
       </c>
-      <c r="E9" s="15" t="s">
+      <c r="E9" s="14" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="17" t="s">
+      <c r="A10" s="16" t="s">
         <v>81</v>
       </c>
-      <c r="D10" s="18" t="n">
+      <c r="D10" s="17" t="n">
         <f aca="false">SUM(D5:D9)</f>
         <v>725727.272727273</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="17" t="s">
+      <c r="B11" s="16" t="s">
         <v>82</v>
       </c>
-      <c r="C11" s="17" t="s">
+      <c r="C11" s="16" t="s">
         <v>83</v>
       </c>
-      <c r="D11" s="17" t="s">
+      <c r="D11" s="16" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="17" t="s">
+      <c r="A12" s="16" t="s">
         <v>85</v>
       </c>
-      <c r="B12" s="16" t="n">
+      <c r="B12" s="15" t="n">
         <v>0.4</v>
       </c>
-      <c r="C12" s="16" t="n">
+      <c r="C12" s="15" t="n">
         <v>0.8</v>
       </c>
-      <c r="D12" s="16" t="n">
+      <c r="D12" s="15" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="14" t="s">
+      <c r="A13" s="13" t="s">
         <v>86</v>
       </c>
-      <c r="B13" s="15" t="s">
+      <c r="B13" s="14" t="s">
         <v>87</v>
       </c>
-      <c r="C13" s="15"/>
-      <c r="D13" s="15"/>
-      <c r="E13" s="15"/>
+      <c r="C13" s="14"/>
+      <c r="D13" s="14"/>
+      <c r="E13" s="14"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1675,233 +1671,233 @@
   <dimension ref="A1:F14"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="3" style="1" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="3" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="52"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="10" t="s">
+      <c r="A2" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="B2" s="10"/>
-      <c r="C2" s="10"/>
-      <c r="D2" s="10"/>
-      <c r="E2" s="10"/>
-      <c r="F2" s="10"/>
+      <c r="B2" s="9"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="11" t="s">
+      <c r="A4" s="10" t="s">
         <v>90</v>
       </c>
-      <c r="B4" s="11" t="s">
+      <c r="B4" s="10" t="s">
         <v>91</v>
       </c>
-      <c r="C4" s="11" t="s">
+      <c r="C4" s="10" t="s">
         <v>82</v>
       </c>
-      <c r="D4" s="11" t="s">
+      <c r="D4" s="10" t="s">
         <v>83</v>
       </c>
-      <c r="E4" s="11" t="s">
+      <c r="E4" s="10" t="s">
         <v>84</v>
       </c>
-      <c r="F4" s="11" t="s">
+      <c r="F4" s="10" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="12" t="s">
+      <c r="A5" s="11" t="s">
         <v>92</v>
       </c>
-      <c r="B5" s="13" t="n">
+      <c r="B5" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="C5" s="13" t="n">
+      <c r="C5" s="12" t="n">
         <v>90000</v>
       </c>
-      <c r="D5" s="13" t="n">
+      <c r="D5" s="12" t="n">
         <v>90000</v>
       </c>
-      <c r="E5" s="13" t="n">
+      <c r="E5" s="12" t="n">
         <v>90000</v>
       </c>
-      <c r="F5" s="15" t="s">
+      <c r="F5" s="14" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="12" t="s">
+      <c r="A6" s="11" t="s">
         <v>94</v>
       </c>
-      <c r="B6" s="13" t="n">
+      <c r="B6" s="12" t="n">
         <v>250000</v>
       </c>
-      <c r="C6" s="13" t="n">
+      <c r="C6" s="12" t="n">
         <v>30000</v>
       </c>
-      <c r="D6" s="13" t="n">
+      <c r="D6" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="E6" s="13" t="n">
+      <c r="E6" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="F6" s="15" t="s">
+      <c r="F6" s="14" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="12" t="s">
+      <c r="A7" s="11" t="s">
         <v>96</v>
       </c>
-      <c r="B7" s="13" t="n">
+      <c r="B7" s="12" t="n">
         <v>80000</v>
       </c>
-      <c r="C7" s="13" t="n">
+      <c r="C7" s="12" t="n">
         <v>10000</v>
       </c>
-      <c r="D7" s="13" t="n">
+      <c r="D7" s="12" t="n">
         <v>10000</v>
       </c>
-      <c r="E7" s="13" t="n">
+      <c r="E7" s="12" t="n">
         <v>10000</v>
       </c>
-      <c r="F7" s="15" t="s">
+      <c r="F7" s="14" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="12" t="s">
+      <c r="A8" s="11" t="s">
         <v>98</v>
       </c>
-      <c r="B8" s="13" t="n">
+      <c r="B8" s="12" t="n">
         <v>60000</v>
       </c>
-      <c r="C8" s="13" t="n">
+      <c r="C8" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="D8" s="13" t="n">
+      <c r="D8" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="E8" s="13" t="n">
+      <c r="E8" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="F8" s="15" t="s">
+      <c r="F8" s="14" t="s">
         <v>99</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="12" t="s">
+      <c r="A9" s="11" t="s">
         <v>100</v>
       </c>
-      <c r="B9" s="13" t="n">
+      <c r="B9" s="12" t="n">
         <v>150000</v>
       </c>
-      <c r="C9" s="13" t="n">
+      <c r="C9" s="12" t="n">
         <v>80000</v>
       </c>
-      <c r="D9" s="13" t="n">
+      <c r="D9" s="12" t="n">
         <v>40000</v>
       </c>
-      <c r="E9" s="13" t="n">
+      <c r="E9" s="12" t="n">
         <v>40000</v>
       </c>
-      <c r="F9" s="15" t="s">
+      <c r="F9" s="14" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="12" t="s">
+      <c r="A10" s="11" t="s">
         <v>102</v>
       </c>
-      <c r="B10" s="13" t="n">
+      <c r="B10" s="12" t="n">
         <v>30000</v>
       </c>
-      <c r="C10" s="13" t="n">
+      <c r="C10" s="12" t="n">
         <v>10000</v>
       </c>
-      <c r="D10" s="13" t="n">
+      <c r="D10" s="12" t="n">
         <v>5000</v>
       </c>
-      <c r="E10" s="13" t="n">
+      <c r="E10" s="12" t="n">
         <v>5000</v>
       </c>
-      <c r="F10" s="15" t="s">
+      <c r="F10" s="14" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="12" t="s">
+      <c r="A11" s="11" t="s">
         <v>104</v>
       </c>
-      <c r="B11" s="13" t="n">
+      <c r="B11" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="C11" s="13" t="n">
+      <c r="C11" s="12" t="n">
         <v>25000</v>
       </c>
-      <c r="D11" s="13" t="n">
+      <c r="D11" s="12" t="n">
         <v>25000</v>
       </c>
-      <c r="E11" s="13" t="n">
+      <c r="E11" s="12" t="n">
         <v>25000</v>
       </c>
-      <c r="F11" s="15" t="s">
+      <c r="F11" s="14" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="17" t="s">
+      <c r="A12" s="16" t="s">
         <v>106</v>
       </c>
-      <c r="B12" s="21" t="n">
+      <c r="B12" s="20" t="n">
         <f aca="false">SUM(B5:B11)*$B$13</f>
         <v>85500</v>
       </c>
-      <c r="C12" s="21" t="n">
+      <c r="C12" s="20" t="n">
         <f aca="false">SUM(C5:C11)*$B$13</f>
         <v>36750</v>
       </c>
-      <c r="D12" s="21" t="n">
+      <c r="D12" s="20" t="n">
         <f aca="false">SUM(D5:D11)*$B$13</f>
         <v>25500</v>
       </c>
-      <c r="E12" s="21" t="n">
+      <c r="E12" s="20" t="n">
         <f aca="false">SUM(E5:E11)*$B$13</f>
         <v>25500</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="12" t="s">
+      <c r="A13" s="11" t="s">
         <v>107</v>
       </c>
-      <c r="B13" s="16" t="n">
+      <c r="B13" s="15" t="n">
         <v>0.15</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="17" t="s">
+      <c r="A14" s="16" t="s">
         <v>108</v>
       </c>
-      <c r="B14" s="18" t="n">
+      <c r="B14" s="17" t="n">
         <f aca="false">SUM(B5:B12)</f>
         <v>655500</v>
       </c>
-      <c r="C14" s="18" t="n">
+      <c r="C14" s="17" t="n">
         <f aca="false">SUM(C5:C12)</f>
         <v>281750</v>
       </c>
-      <c r="D14" s="18" t="n">
+      <c r="D14" s="17" t="n">
         <f aca="false">SUM(D5:D12)</f>
         <v>195500</v>
       </c>
-      <c r="E14" s="18" t="n">
+      <c r="E14" s="17" t="n">
         <f aca="false">SUM(E5:E12)</f>
         <v>195500</v>
       </c>
@@ -1929,177 +1925,177 @@
   <dimension ref="A1:F16"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="2" style="1" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="2" style="0" width="15"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="10" t="s">
+      <c r="A2" s="9" t="s">
         <v>110</v>
       </c>
-      <c r="B2" s="10"/>
-      <c r="C2" s="10"/>
-      <c r="D2" s="10"/>
-      <c r="E2" s="10"/>
-      <c r="F2" s="10"/>
+      <c r="B2" s="9"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="11"/>
-      <c r="B4" s="11" t="s">
+      <c r="A4" s="10"/>
+      <c r="B4" s="10" t="s">
         <v>111</v>
       </c>
-      <c r="C4" s="11" t="s">
+      <c r="C4" s="10" t="s">
         <v>82</v>
       </c>
-      <c r="D4" s="11" t="s">
+      <c r="D4" s="10" t="s">
         <v>83</v>
       </c>
-      <c r="E4" s="11" t="s">
+      <c r="E4" s="10" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="12" t="s">
+      <c r="A5" s="11" t="s">
         <v>112</v>
       </c>
-      <c r="B5" s="21" t="n">
+      <c r="B5" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="C5" s="20" t="n">
+      <c r="C5" s="19" t="n">
         <f aca="false">Benefits!$D$10*Benefits!B12</f>
         <v>290290.909090909</v>
       </c>
-      <c r="D5" s="20" t="n">
+      <c r="D5" s="19" t="n">
         <f aca="false">Benefits!$D$10*Benefits!C12</f>
         <v>580581.818181818</v>
       </c>
-      <c r="E5" s="20" t="n">
+      <c r="E5" s="19" t="n">
         <f aca="false">Benefits!$D$10*Benefits!D12</f>
         <v>725727.272727273</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="12" t="s">
+      <c r="A6" s="11" t="s">
         <v>113</v>
       </c>
-      <c r="B6" s="20" t="n">
+      <c r="B6" s="19" t="n">
         <f aca="false">-Costs!B14</f>
         <v>-655500</v>
       </c>
-      <c r="C6" s="20" t="n">
+      <c r="C6" s="19" t="n">
         <f aca="false">-Costs!C14</f>
         <v>-281750</v>
       </c>
-      <c r="D6" s="20" t="n">
+      <c r="D6" s="19" t="n">
         <f aca="false">-Costs!D14</f>
         <v>-195500</v>
       </c>
-      <c r="E6" s="20" t="n">
+      <c r="E6" s="19" t="n">
         <f aca="false">-Costs!E14</f>
         <v>-195500</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="17" t="s">
+      <c r="A7" s="16" t="s">
         <v>114</v>
       </c>
-      <c r="B7" s="22" t="n">
+      <c r="B7" s="21" t="n">
         <f aca="false">B5+B6</f>
         <v>-655500</v>
       </c>
-      <c r="C7" s="22" t="n">
+      <c r="C7" s="21" t="n">
         <f aca="false">C5+C6</f>
         <v>8540.90909090912</v>
       </c>
-      <c r="D7" s="22" t="n">
+      <c r="D7" s="21" t="n">
         <f aca="false">D5+D6</f>
         <v>385081.818181818</v>
       </c>
-      <c r="E7" s="22" t="n">
+      <c r="E7" s="21" t="n">
         <f aca="false">E5+E6</f>
         <v>530227.272727273</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="17" t="s">
+      <c r="A8" s="16" t="s">
         <v>115</v>
       </c>
-      <c r="B8" s="18" t="n">
+      <c r="B8" s="17" t="n">
         <f aca="false">B7</f>
         <v>-655500</v>
       </c>
-      <c r="C8" s="18" t="n">
+      <c r="C8" s="17" t="n">
         <f aca="false">B8+C7</f>
         <v>-646959.090909091</v>
       </c>
-      <c r="D8" s="18" t="n">
+      <c r="D8" s="17" t="n">
         <f aca="false">C8+D7</f>
         <v>-261877.272727273</v>
       </c>
-      <c r="E8" s="18" t="n">
+      <c r="E8" s="17" t="n">
         <f aca="false">D8+E7</f>
         <v>268350</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="17" t="s">
+      <c r="A10" s="16" t="s">
         <v>116</v>
       </c>
-      <c r="B10" s="22" t="n">
+      <c r="B10" s="21" t="n">
         <f aca="false">SUM(C5:E5)</f>
         <v>1596600</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="17" t="s">
+      <c r="A11" s="16" t="s">
         <v>117</v>
       </c>
-      <c r="B11" s="22" t="n">
+      <c r="B11" s="21" t="n">
         <f aca="false">-SUM(B6:E6)</f>
         <v>1328250</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="17" t="s">
+      <c r="A12" s="16" t="s">
         <v>118</v>
       </c>
-      <c r="B12" s="18" t="n">
+      <c r="B12" s="17" t="n">
         <f aca="false">B10-B11</f>
         <v>268350</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="17" t="s">
+      <c r="A13" s="16" t="s">
         <v>119</v>
       </c>
-      <c r="B13" s="23" t="n">
+      <c r="B13" s="22" t="n">
         <f aca="false">IF(B11&gt;0,B12/B11,0)</f>
         <v>0.202032749858837</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="17" t="s">
+      <c r="A14" s="16" t="s">
         <v>120</v>
       </c>
-      <c r="B14" s="24" t="str">
+      <c r="B14" s="23" t="str">
         <f aca="false">IF(C8&gt;=0,"Year 1",IF(D8&gt;=0,"Year 2",IF(E8&gt;=0,"Year 3","After year 3")))</f>
         <v>Year 3</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="17" t="s">
+      <c r="A16" s="16" t="s">
         <v>121</v>
       </c>
-      <c r="B16" s="20" t="n">
+      <c r="B16" s="19" t="n">
         <f aca="false">Benefits!D10</f>
         <v>725727.272727273</v>
       </c>
-      <c r="C16" s="14" t="s">
+      <c r="C16" s="13" t="s">
         <v>122</v>
       </c>
     </row>
@@ -2131,132 +2127,132 @@
   <dimension ref="A1:F10"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="36"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="20"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>123</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="10" t="s">
+      <c r="A2" s="9" t="s">
         <v>124</v>
       </c>
-      <c r="B2" s="10"/>
-      <c r="C2" s="10"/>
-      <c r="D2" s="10"/>
-      <c r="E2" s="10"/>
-      <c r="F2" s="10"/>
+      <c r="B2" s="9"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="11" t="s">
+      <c r="A4" s="10" t="s">
         <v>125</v>
       </c>
-      <c r="B4" s="11" t="s">
+      <c r="B4" s="10" t="s">
         <v>126</v>
       </c>
-      <c r="C4" s="11" t="s">
+      <c r="C4" s="10" t="s">
         <v>127</v>
       </c>
-      <c r="D4" s="11" t="s">
+      <c r="D4" s="10" t="s">
         <v>128</v>
       </c>
-      <c r="E4" s="11" t="s">
+      <c r="E4" s="10" t="s">
         <v>129</v>
       </c>
-      <c r="F4" s="11" t="s">
+      <c r="F4" s="10" t="s">
         <v>130</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="25" t="s">
+      <c r="A5" s="24" t="s">
         <v>131</v>
       </c>
-      <c r="B5" s="25" t="s">
+      <c r="B5" s="24" t="s">
         <v>132</v>
       </c>
-      <c r="C5" s="25" t="s">
+      <c r="C5" s="24" t="s">
         <v>133</v>
       </c>
-      <c r="D5" s="25" t="s">
+      <c r="D5" s="24" t="s">
         <v>134</v>
       </c>
-      <c r="E5" s="25" t="s">
+      <c r="E5" s="24" t="s">
         <v>135</v>
       </c>
-      <c r="F5" s="25" t="s">
+      <c r="F5" s="24" t="s">
         <v>136</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="25" t="s">
+      <c r="A6" s="24" t="s">
         <v>137</v>
       </c>
-      <c r="B6" s="25" t="s">
+      <c r="B6" s="24" t="s">
         <v>138</v>
       </c>
-      <c r="C6" s="25" t="s">
+      <c r="C6" s="24" t="s">
         <v>139</v>
       </c>
-      <c r="D6" s="25" t="s">
+      <c r="D6" s="24" t="s">
         <v>140</v>
       </c>
-      <c r="E6" s="25" t="s">
+      <c r="E6" s="24" t="s">
         <v>141</v>
       </c>
-      <c r="F6" s="25" t="s">
+      <c r="F6" s="24" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="25" t="s">
+      <c r="A7" s="24" t="s">
         <v>143</v>
       </c>
-      <c r="B7" s="25" t="s">
+      <c r="B7" s="24" t="s">
         <v>144</v>
       </c>
-      <c r="C7" s="25" t="s">
+      <c r="C7" s="24" t="s">
+        <v>133</v>
+      </c>
+      <c r="D7" s="24" t="s">
         <v>145</v>
       </c>
-      <c r="D7" s="25" t="s">
+      <c r="E7" s="24" t="s">
         <v>146</v>
       </c>
-      <c r="E7" s="25" t="s">
+      <c r="F7" s="24" t="s">
         <v>147</v>
       </c>
-      <c r="F7" s="25" t="s">
-        <v>142</v>
-      </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="26"/>
-      <c r="B8" s="26"/>
-      <c r="C8" s="26"/>
-      <c r="D8" s="26"/>
-      <c r="E8" s="26"/>
-      <c r="F8" s="26"/>
+      <c r="A8" s="25"/>
+      <c r="B8" s="25"/>
+      <c r="C8" s="25"/>
+      <c r="D8" s="25"/>
+      <c r="E8" s="25"/>
+      <c r="F8" s="25"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="26"/>
-      <c r="B9" s="26"/>
-      <c r="C9" s="26"/>
-      <c r="D9" s="26"/>
-      <c r="E9" s="26"/>
-      <c r="F9" s="26"/>
+      <c r="A9" s="25"/>
+      <c r="B9" s="25"/>
+      <c r="C9" s="25"/>
+      <c r="D9" s="25"/>
+      <c r="E9" s="25"/>
+      <c r="F9" s="25"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="26"/>
-      <c r="B10" s="26"/>
-      <c r="C10" s="26"/>
-      <c r="D10" s="26"/>
-      <c r="E10" s="26"/>
-      <c r="F10" s="26"/>
+      <c r="A10" s="25"/>
+      <c r="B10" s="25"/>
+      <c r="C10" s="25"/>
+      <c r="D10" s="25"/>
+      <c r="E10" s="25"/>
+      <c r="F10" s="25"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Strategic, company-wide decision with phased delivery: unreviewed pages, how-long article, business case template
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Y4SNSUs71veJ37BenGhXFE
</commit_message>
<xml_diff>
--- a/public/downloads/shopfloor-matters-business-case-template.xlsx
+++ b/public/downloads/shopfloor-matters-business-case-template.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Benefits" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="Costs" sheetId="4" state="visible" r:id="rId6"/>
     <sheet name="Cash flow" sheetId="5" state="visible" r:id="rId7"/>
-    <sheet name="Phasing" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="Rollout plan" sheetId="6" state="visible" r:id="rId8"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -64,7 +64,7 @@
     <t xml:space="preserve">3. Realistic costs and timeline, including your own people, not just licences and services (Costs).</t>
   </si>
   <si>
-    <t xml:space="preserve">4. How the risk is managed: phases, measures and decision points (Phasing).</t>
+    <t xml:space="preserve">4. How the risk is managed: a phased rollout plan with measures and milestones (Rollout plan).</t>
   </si>
   <si>
     <t xml:space="preserve">How to use it:</t>
@@ -73,7 +73,7 @@
     <t xml:space="preserve">Fill in Baseline with numbers finance will recognise. Set deliberately modest improvements on Benefits. Fill in every cost line, then read Cash flow.</t>
   </si>
   <si>
-    <t xml:space="preserve">Keep the first phase small: one line or one area. Let its results fund the next phase.</t>
+    <t xml:space="preserve">Make the decision once, for the whole programme, then phase the delivery: by function, by site, or both.</t>
   </si>
   <si>
     <t xml:space="preserve">The example values describe a fictional mid-size site so you can see how it works. They are not a forecast. Replace them all.</t>
@@ -418,10 +418,10 @@
     <t xml:space="preserve">Every year you wait, this is what stays on the table.</t>
   </si>
   <si>
-    <t xml:space="preserve">Phasing: how the risk is managed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The section boards read most closely. Each phase has a scope, a measure and a decision point. The next phase only starts when the measure says so.</t>
+    <t xml:space="preserve">Rollout plan: how the risk is managed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The section boards read most closely. The decision covers the whole programme. Each phase has a scope, a measure and a milestone, so progress is visible all the way.</t>
   </si>
   <si>
     <t xml:space="preserve">Phase</t>
@@ -436,61 +436,61 @@
     <t xml:space="preserve">Success measure</t>
   </si>
   <si>
-    <t xml:space="preserve">Decision point</t>
+    <t xml:space="preserve">Milestone</t>
   </si>
   <si>
     <t xml:space="preserve">Owner</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Pilot</t>
-  </si>
-  <si>
-    <t xml:space="preserve">One line, production and quality</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4 to 6 months</t>
+    <t xml:space="preserve">1. Production and quality</t>
+  </si>
+  <si>
+    <t xml:space="preserve">First sites in the rollout plan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6 to 9 months</t>
   </si>
   <si>
     <t xml:space="preserve">OEE up 3 points against baseline; scrap down 10%</t>
   </si>
   <si>
-    <t xml:space="preserve">Steering group review at month 6</t>
+    <t xml:space="preserve">Live on every shift at the first sites</t>
   </si>
   <si>
     <t xml:space="preserve">Operations director</t>
   </si>
   <si>
-    <t xml:space="preserve">2. Site</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Remaining lines on the site</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6 to 9 months</t>
+    <t xml:space="preserve">2. Remaining sites</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Production and quality at every other site, from the template</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12 to 24 months</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Go-live on time with under 10% local change</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Each site live on every shift</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Programme lead</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3. Inventory and maintenance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Switched on across every site</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6 to 12 months</t>
   </si>
   <si>
     <t xml:space="preserve">Benefits on Benefits sheet reached at 80% ramp</t>
   </si>
   <si>
-    <t xml:space="preserve">Before committing to site 2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Site lead</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3. Template</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Second site from the same template</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Go-live on time with under 10% local change</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Before wider roll-out</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Programme lead</t>
+    <t xml:space="preserve">Live at every site</t>
   </si>
 </sst>
 </file>
@@ -1123,7 +1123,7 @@
       <c r="G9" s="3"/>
       <c r="H9" s="3"/>
     </row>
-    <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
         <v>8</v>
       </c>
@@ -2218,16 +2218,16 @@
         <v>144</v>
       </c>
       <c r="C7" s="24" t="s">
-        <v>133</v>
+        <v>145</v>
       </c>
       <c r="D7" s="24" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E7" s="24" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F7" s="24" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>